<commit_message>
Upload Week 2-6 lengkap
</commit_message>
<xml_diff>
--- a/Week 5/week 5 - Cara Kerja KNN Eucadian Rumus.xlsx
+++ b/Week 5/week 5 - Cara Kerja KNN Eucadian Rumus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yosua Dirgana\Downloads\File Semester 6\Machine Learning\Github Yosua\Week 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABB0EA4-6CE0-4B30-85BE-6DD8B6C98542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8507F01-3629-4B71-838A-9074D97D842A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{616F7598-4A7E-4CBD-AA13-0B6816B444CE}"/>
   </bookViews>
@@ -432,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -445,14 +445,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -466,6 +460,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2707,16 +2704,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>218534</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>152348</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>134</xdr:row>
+      <xdr:rowOff>18998</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>475198</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>176593</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>104264</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>43243</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2745,16 +2742,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>185531</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>171</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>112</xdr:row>
-      <xdr:rowOff>138319</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>271669</xdr:colOff>
+      <xdr:row>184</xdr:row>
+      <xdr:rowOff>62119</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2769,8 +2766,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3378311" y="18966180"/>
-          <a:ext cx="4081669" cy="2287159"/>
+          <a:off x="0" y="33497520"/>
+          <a:ext cx="4081669" cy="2378599"/>
           <a:chOff x="3459977" y="18908924"/>
           <a:chExt cx="4545496" cy="2636520"/>
         </a:xfrm>
@@ -4142,89 +4139,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F963C0-90C0-49A8-9F06-162F25B885A3}">
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="14"/>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13">
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11">
         <v>4222301009</v>
       </c>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H4" t="s">
-        <v>1</v>
-      </c>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="H6" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -4240,22 +4209,6 @@
       <c r="D9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="5">
-        <v>7</v>
-      </c>
-      <c r="I9" s="5">
-        <v>7</v>
-      </c>
-      <c r="J9" s="5">
-        <v>4</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L9" s="6">
-        <f>SQRT((I9-6)^2 + (J9-5)^2)</f>
-        <v>1.4142135623730951</v>
-      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
@@ -4270,22 +4223,6 @@
       <c r="D10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H10" s="5">
-        <v>6</v>
-      </c>
-      <c r="I10" s="5">
-        <v>6</v>
-      </c>
-      <c r="J10" s="5">
-        <v>3</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L10" s="6">
-        <f>SQRT((I10-6)^2 + (J10-5)^2)</f>
-        <v>2</v>
-      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
@@ -4300,22 +4237,6 @@
       <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="5">
-        <v>5</v>
-      </c>
-      <c r="I11" s="5">
-        <v>5</v>
-      </c>
-      <c r="J11" s="5">
-        <v>3</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L11" s="6">
-        <f>SQRT((I11-6)^2 + (J11-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
@@ -4330,22 +4251,6 @@
       <c r="D12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="5">
-        <v>8</v>
-      </c>
-      <c r="I12" s="5">
-        <v>8</v>
-      </c>
-      <c r="J12" s="5">
-        <v>4</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L12" s="6">
-        <f>SQRT((I12-6)^2 + (J12-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
@@ -4360,22 +4265,6 @@
       <c r="D13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="5">
-        <v>14</v>
-      </c>
-      <c r="I13" s="5">
-        <v>4</v>
-      </c>
-      <c r="J13" s="5">
-        <v>7</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L13" s="6">
-        <f>SQRT((I13-6)^2 + (J13-5)^2)</f>
-        <v>2.8284271247461903</v>
-      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
@@ -4390,22 +4279,6 @@
       <c r="D14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="5">
-        <v>9</v>
-      </c>
-      <c r="I14" s="5">
-        <v>9</v>
-      </c>
-      <c r="J14" s="5">
-        <v>5</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L14" s="6">
-        <f>SQRT((I14-6)^2 + (J14-5)^2)</f>
-        <v>3</v>
-      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
@@ -4420,22 +4293,6 @@
       <c r="D15" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="5">
-        <v>16</v>
-      </c>
-      <c r="I15" s="5">
-        <v>6</v>
-      </c>
-      <c r="J15" s="5">
-        <v>8</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L15" s="6">
-        <f>SQRT((I15-6)^2 + (J15-5)^2)</f>
-        <v>3</v>
-      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
@@ -4450,24 +4307,8 @@
       <c r="D16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="5">
-        <v>15</v>
-      </c>
-      <c r="I16" s="5">
-        <v>5</v>
-      </c>
-      <c r="J16" s="5">
-        <v>8</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L16" s="6">
-        <f>SQRT((I16-6)^2 + (J16-5)^2)</f>
-        <v>3.1622776601683795</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>8</v>
       </c>
@@ -4480,24 +4321,8 @@
       <c r="D17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H17" s="5">
-        <v>4</v>
-      </c>
-      <c r="I17" s="5">
-        <v>4</v>
-      </c>
-      <c r="J17" s="5">
-        <v>2</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L17" s="6">
-        <f>SQRT((I17-6)^2 + (J17-5)^2)</f>
-        <v>3.6055512754639891</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>9</v>
       </c>
@@ -4510,24 +4335,8 @@
       <c r="D18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H18" s="5">
-        <v>13</v>
-      </c>
-      <c r="I18" s="5">
-        <v>3</v>
-      </c>
-      <c r="J18" s="5">
-        <v>7</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L18" s="6">
-        <f>SQRT((I18-6)^2 + (J18-5)^2)</f>
-        <v>3.6055512754639891</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>10</v>
       </c>
@@ -4540,24 +4349,8 @@
       <c r="D19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="5">
-        <v>10</v>
-      </c>
-      <c r="I19" s="5">
-        <v>10</v>
-      </c>
-      <c r="J19" s="5">
-        <v>5</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L19" s="6">
-        <f>SQRT((I19-6)^2 + (J19-5)^2)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <v>11</v>
       </c>
@@ -4570,24 +4363,8 @@
       <c r="D20" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="5">
-        <v>12</v>
-      </c>
-      <c r="I20" s="5">
-        <v>2</v>
-      </c>
-      <c r="J20" s="5">
-        <v>6</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L20" s="6">
-        <f>SQRT((I20-6)^2 + (J20-5)^2)</f>
-        <v>4.1231056256176606</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>12</v>
       </c>
@@ -4600,24 +4377,8 @@
       <c r="D21" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H21" s="5">
-        <v>17</v>
-      </c>
-      <c r="I21" s="5">
-        <v>7</v>
-      </c>
-      <c r="J21" s="5">
-        <v>9</v>
-      </c>
-      <c r="K21" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L21" s="6">
-        <f>SQRT((I21-6)^2 + (J21-5)^2)</f>
-        <v>4.1231056256176606</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>13</v>
       </c>
@@ -4630,24 +4391,8 @@
       <c r="D22" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H22" s="5">
-        <v>3</v>
-      </c>
-      <c r="I22" s="5">
-        <v>3</v>
-      </c>
-      <c r="J22" s="5">
-        <v>2</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L22" s="6">
-        <f>SQRT((I22-6)^2 + (J22-5)^2)</f>
-        <v>4.2426406871192848</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>14</v>
       </c>
@@ -4660,24 +4405,8 @@
       <c r="D23" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H23" s="5">
-        <v>18</v>
-      </c>
-      <c r="I23" s="5">
-        <v>8</v>
-      </c>
-      <c r="J23" s="5">
-        <v>9</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L23" s="6">
-        <f>SQRT((I23-6)^2 + (J23-5)^2)</f>
-        <v>4.4721359549995796</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
         <v>15</v>
       </c>
@@ -4690,24 +4419,8 @@
       <c r="D24" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="5">
-        <v>11</v>
-      </c>
-      <c r="I24" s="5">
-        <v>1</v>
-      </c>
-      <c r="J24" s="5">
-        <v>6</v>
-      </c>
-      <c r="K24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L24" s="6">
-        <f>SQRT((I24-6)^2 + (J24-5)^2)</f>
-        <v>5.0990195135927845</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>16</v>
       </c>
@@ -4720,24 +4433,8 @@
       <c r="D25" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="5">
-        <v>2</v>
-      </c>
-      <c r="I25" s="5">
-        <v>2</v>
-      </c>
-      <c r="J25" s="5">
-        <v>1</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L25" s="6">
-        <f>SQRT((I25-6)^2 + (J25-5)^2)</f>
-        <v>5.6568542494923806</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
         <v>17</v>
       </c>
@@ -4750,24 +4447,8 @@
       <c r="D26" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H26" s="5">
-        <v>19</v>
-      </c>
-      <c r="I26" s="5">
-        <v>9</v>
-      </c>
-      <c r="J26" s="5">
-        <v>10</v>
-      </c>
-      <c r="K26" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="L26" s="6">
-        <f>SQRT((I26-6)^2 + (J26-5)^2)</f>
-        <v>5.8309518948453007</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
         <v>18</v>
       </c>
@@ -4780,24 +4461,8 @@
       <c r="D27" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H27" s="5">
-        <v>1</v>
-      </c>
-      <c r="I27" s="5">
-        <v>1</v>
-      </c>
-      <c r="J27" s="5">
-        <v>1</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L27" s="6">
-        <f>SQRT((I27-6)^2 + (J27-5)^2)</f>
-        <v>6.4031242374328485</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
         <v>19</v>
       </c>
@@ -4810,24 +4475,8 @@
       <c r="D28" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H28" s="5">
-        <v>20</v>
-      </c>
-      <c r="I28" s="5">
-        <v>10</v>
-      </c>
-      <c r="J28" s="5">
-        <v>10</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L28" s="6">
-        <f>SQRT((I28-6)^2 + (J28-5)^2)</f>
-        <v>6.4031242374328485</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
         <v>20</v>
       </c>
@@ -4841,254 +4490,206 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="I30" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="5">
+        <v>7</v>
+      </c>
+      <c r="B36" s="5">
+        <v>7</v>
+      </c>
+      <c r="C36" s="5">
+        <v>4</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="7">
+        <f>SQRT((B36-6)^2 + (C36-5)^2)</f>
+        <v>1.4142135623730951</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="5">
+        <v>6</v>
+      </c>
+      <c r="B37" s="5">
+        <v>6</v>
+      </c>
+      <c r="C37" s="5">
+        <v>3</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="7">
+        <f>SQRT((B37-6)^2 + (C37-5)^2)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="5">
+        <v>5</v>
+      </c>
+      <c r="B38" s="5">
+        <v>5</v>
+      </c>
+      <c r="C38" s="5">
+        <v>3</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="7">
+        <f>SQRT((B38-6)^2 + (C38-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="5">
+        <v>8</v>
+      </c>
+      <c r="B39" s="5">
+        <v>8</v>
+      </c>
+      <c r="C39" s="5">
+        <v>4</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="7">
+        <f>SQRT((B39-6)^2 + (C39-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="5">
+        <v>14</v>
+      </c>
+      <c r="B40" s="5">
+        <v>4</v>
+      </c>
+      <c r="C40" s="5">
+        <v>7</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="7">
+        <f>SQRT((B40-6)^2 + (C40-5)^2)</f>
+        <v>2.8284271247461903</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="5">
+        <v>9</v>
+      </c>
+      <c r="B41" s="5">
+        <v>9</v>
+      </c>
+      <c r="C41" s="5">
+        <v>5</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="7">
+        <f>SQRT((B41-6)^2 + (C41-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="5">
+        <v>16</v>
+      </c>
+      <c r="B42" s="5">
+        <v>6</v>
+      </c>
+      <c r="C42" s="5">
+        <v>8</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" s="7">
+        <f>SQRT((B42-6)^2 + (C42-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="5">
+        <v>15</v>
+      </c>
+      <c r="B43" s="5">
+        <v>5</v>
+      </c>
+      <c r="C43" s="5">
+        <v>8</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="7">
+        <f>SQRT((B43-6)^2 + (C43-5)^2)</f>
+        <v>3.1622776601683795</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="5">
+        <v>4</v>
+      </c>
+      <c r="B44" s="5">
+        <v>4</v>
+      </c>
+      <c r="C44" s="5">
+        <v>2</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" s="7">
+        <f>SQRT((B44-6)^2 + (C44-5)^2)</f>
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="5">
         <v>13</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>14</v>
-      </c>
-      <c r="I32" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>17</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="11"/>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>18</v>
-      </c>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-      <c r="N34" s="11"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>20</v>
-      </c>
-      <c r="I36" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>21</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="K38" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J40" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="L40" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="M40" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="8">
-        <v>7</v>
-      </c>
-      <c r="B41" s="8">
-        <v>7</v>
-      </c>
-      <c r="C41" s="8">
-        <v>4</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" s="9">
-        <f>SQRT((B41-6)^2 + (C41-5)^2)</f>
-        <v>1.4142135623730951</v>
-      </c>
-      <c r="I41" s="8">
-        <v>7</v>
-      </c>
-      <c r="J41" s="8">
-        <v>7</v>
-      </c>
-      <c r="K41" s="8">
-        <v>4</v>
-      </c>
-      <c r="L41" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="M41" s="9">
-        <f>SQRT((J41-6)^2 + (K41-5)^2)</f>
-        <v>1.4142135623730951</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="8">
-        <v>6</v>
-      </c>
-      <c r="B42" s="8">
-        <v>6</v>
-      </c>
-      <c r="C42" s="8">
+      <c r="B45" s="5">
         <v>3</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E42" s="9">
-        <f>SQRT((B42-6)^2 + (C42-5)^2)</f>
-        <v>2</v>
-      </c>
-      <c r="I42" s="8">
-        <v>6</v>
-      </c>
-      <c r="J42" s="8">
-        <v>6</v>
-      </c>
-      <c r="K42" s="8">
-        <v>3</v>
-      </c>
-      <c r="L42" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="M42" s="9">
-        <f>SQRT((J42-6)^2 + (K42-5)^2)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="8">
-        <v>5</v>
-      </c>
-      <c r="B43" s="8">
-        <v>5</v>
-      </c>
-      <c r="C43" s="8">
-        <v>3</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" s="9">
-        <f>SQRT((B43-6)^2 + (C43-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-      <c r="I43" s="8">
-        <v>5</v>
-      </c>
-      <c r="J43" s="8">
-        <v>5</v>
-      </c>
-      <c r="K43" s="8">
-        <v>3</v>
-      </c>
-      <c r="L43" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="M43" s="9">
-        <f>SQRT((J43-6)^2 + (K43-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="8">
-        <v>8</v>
-      </c>
-      <c r="B44" s="8">
-        <v>8</v>
-      </c>
-      <c r="C44" s="8">
-        <v>4</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E44" s="9">
-        <f>SQRT((B44-6)^2 + (C44-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-      <c r="I44" s="8">
-        <v>8</v>
-      </c>
-      <c r="J44" s="8">
-        <v>8</v>
-      </c>
-      <c r="K44" s="8">
-        <v>4</v>
-      </c>
-      <c r="L44" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="M44" s="9">
-        <f>SQRT((J44-6)^2 + (K44-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="5">
-        <v>14</v>
-      </c>
-      <c r="B45" s="5">
-        <v>4</v>
       </c>
       <c r="C45" s="5">
         <v>7</v>
@@ -5096,912 +4697,786 @@
       <c r="D45" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="7">
         <f>SQRT((B45-6)^2 + (C45-5)^2)</f>
-        <v>2.8284271247461903</v>
-      </c>
-      <c r="I45" s="8">
-        <v>9</v>
-      </c>
-      <c r="J45" s="8">
-        <v>9</v>
-      </c>
-      <c r="K45" s="8">
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="5">
+        <v>10</v>
+      </c>
+      <c r="B46" s="5">
+        <v>10</v>
+      </c>
+      <c r="C46" s="5">
         <v>5</v>
       </c>
-      <c r="L45" s="8" t="s">
+      <c r="D46" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="7">
+        <f>SQRT((B46-6)^2 + (C46-5)^2)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="5">
         <v>12</v>
       </c>
-      <c r="M45" s="9">
-        <f>SQRT((J45-6)^2 + (K45-5)^2)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="8">
-        <v>9</v>
-      </c>
-      <c r="B46" s="8">
-        <v>9</v>
-      </c>
-      <c r="C46" s="8">
-        <v>5</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E46" s="9">
-        <f>SQRT((B46-6)^2 + (C46-5)^2)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="5">
-        <v>16</v>
-      </c>
       <c r="B47" s="5">
+        <v>2</v>
+      </c>
+      <c r="C47" s="5">
         <v>6</v>
-      </c>
-      <c r="C47" s="5">
-        <v>8</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="7">
         <f>SQRT((B47-6)^2 + (C47-5)^2)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+        <v>4.1231056256176606</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="5">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B48" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C48" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" s="9">
+        <v>11</v>
+      </c>
+      <c r="E48" s="7">
         <f>SQRT((B48-6)^2 + (C48-5)^2)</f>
-        <v>3.1622776601683795</v>
+        <v>4.1231056256176606</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B49" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" s="5">
         <v>2</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E49" s="9">
+        <v>11</v>
+      </c>
+      <c r="E49" s="7">
         <f>SQRT((B49-6)^2 + (C49-5)^2)</f>
-        <v>3.6055512754639891</v>
+        <v>4.2426406871192848</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="5">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B50" s="5">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C50" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E50" s="7">
         <f>SQRT((B50-6)^2 + (C50-5)^2)</f>
-        <v>3.6055512754639891</v>
+        <v>4.4721359549995796</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B51" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C51" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="9">
+        <v>12</v>
+      </c>
+      <c r="E51" s="7">
         <f>SQRT((B51-6)^2 + (C51-5)^2)</f>
-        <v>4</v>
+        <v>5.0990195135927845</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B52" s="5">
         <v>2</v>
       </c>
       <c r="C52" s="5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E52" s="9">
+        <v>11</v>
+      </c>
+      <c r="E52" s="7">
         <f>SQRT((B52-6)^2 + (C52-5)^2)</f>
-        <v>4.1231056256176606</v>
+        <v>5.6568542494923806</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="5">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B53" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C53" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="9">
+        <v>12</v>
+      </c>
+      <c r="E53" s="7">
         <f>SQRT((B53-6)^2 + (C53-5)^2)</f>
-        <v>4.1231056256176606</v>
+        <v>5.8309518948453007</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B54" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C54" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="7">
         <f>SQRT((B54-6)^2 + (C54-5)^2)</f>
-        <v>4.2426406871192848</v>
+        <v>6.4031242374328485</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="5">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B55" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C55" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E55" s="7">
         <f>SQRT((B55-6)^2 + (C55-5)^2)</f>
+        <v>6.4031242374328485</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" s="13">
+        <v>7</v>
+      </c>
+      <c r="B69" s="13">
+        <v>7</v>
+      </c>
+      <c r="C69" s="13">
+        <v>4</v>
+      </c>
+      <c r="D69" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" s="7">
+        <f>SQRT((B69-6)^2 + (C69-5)^2)</f>
+        <v>1.4142135623730951</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" s="13">
+        <v>6</v>
+      </c>
+      <c r="B70" s="13">
+        <v>6</v>
+      </c>
+      <c r="C70" s="13">
+        <v>3</v>
+      </c>
+      <c r="D70" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" s="7">
+        <f>SQRT((B70-6)^2 + (C70-5)^2)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A71" s="13">
+        <v>5</v>
+      </c>
+      <c r="B71" s="13">
+        <v>5</v>
+      </c>
+      <c r="C71" s="13">
+        <v>3</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" s="7">
+        <f>SQRT((B71-6)^2 + (C71-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A72" s="13">
+        <v>8</v>
+      </c>
+      <c r="B72" s="13">
+        <v>8</v>
+      </c>
+      <c r="C72" s="13">
+        <v>4</v>
+      </c>
+      <c r="D72" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E72" s="7">
+        <f>SQRT((B72-6)^2 + (C72-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A73" s="13">
+        <v>14</v>
+      </c>
+      <c r="B73" s="13">
+        <v>4</v>
+      </c>
+      <c r="C73" s="13">
+        <v>7</v>
+      </c>
+      <c r="D73" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" s="7">
+        <f>SQRT((B73-6)^2 + (C73-5)^2)</f>
+        <v>2.8284271247461903</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" s="13">
+        <v>9</v>
+      </c>
+      <c r="B74" s="13">
+        <v>9</v>
+      </c>
+      <c r="C74" s="13">
+        <v>5</v>
+      </c>
+      <c r="D74" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E74" s="7">
+        <f>SQRT((B74-6)^2 + (C74-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A75" s="13">
+        <v>16</v>
+      </c>
+      <c r="B75" s="13">
+        <v>6</v>
+      </c>
+      <c r="C75" s="13">
+        <v>8</v>
+      </c>
+      <c r="D75" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E75" s="7">
+        <f>SQRT((B75-6)^2 + (C75-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" s="13">
+        <v>15</v>
+      </c>
+      <c r="B76" s="13">
+        <v>5</v>
+      </c>
+      <c r="C76" s="13">
+        <v>8</v>
+      </c>
+      <c r="D76" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E76" s="7">
+        <f>SQRT((B76-6)^2 + (C76-5)^2)</f>
+        <v>3.1622776601683795</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A77" s="13">
+        <v>4</v>
+      </c>
+      <c r="B77" s="13">
+        <v>4</v>
+      </c>
+      <c r="C77" s="13">
+        <v>2</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E77" s="7">
+        <f>SQRT((B77-6)^2 + (C77-5)^2)</f>
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A78" s="13">
+        <v>13</v>
+      </c>
+      <c r="B78" s="13">
+        <v>3</v>
+      </c>
+      <c r="C78" s="13">
+        <v>7</v>
+      </c>
+      <c r="D78" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E78" s="7">
+        <f>SQRT((B78-6)^2 + (C78-5)^2)</f>
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" s="13">
+        <v>10</v>
+      </c>
+      <c r="B79" s="13">
+        <v>10</v>
+      </c>
+      <c r="C79" s="13">
+        <v>5</v>
+      </c>
+      <c r="D79" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E79" s="7">
+        <f>SQRT((B79-6)^2 + (C79-5)^2)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" s="13">
+        <v>12</v>
+      </c>
+      <c r="B80" s="13">
+        <v>2</v>
+      </c>
+      <c r="C80" s="13">
+        <v>6</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E80" s="7">
+        <f>SQRT((B80-6)^2 + (C80-5)^2)</f>
+        <v>4.1231056256176606</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" s="13">
+        <v>17</v>
+      </c>
+      <c r="B81" s="13">
+        <v>7</v>
+      </c>
+      <c r="C81" s="13">
+        <v>9</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E81" s="7">
+        <f>SQRT((B81-6)^2 + (C81-5)^2)</f>
+        <v>4.1231056256176606</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" s="13">
+        <v>3</v>
+      </c>
+      <c r="B82" s="13">
+        <v>3</v>
+      </c>
+      <c r="C82" s="13">
+        <v>2</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" s="7">
+        <f>SQRT((B82-6)^2 + (C82-5)^2)</f>
+        <v>4.2426406871192848</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" s="13">
+        <v>18</v>
+      </c>
+      <c r="B83" s="13">
+        <v>8</v>
+      </c>
+      <c r="C83" s="13">
+        <v>9</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" s="7">
+        <f>SQRT((B83-6)^2 + (C83-5)^2)</f>
         <v>4.4721359549995796</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="5">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" s="13">
         <v>11</v>
       </c>
-      <c r="B56" s="5">
+      <c r="B84" s="13">
         <v>1</v>
       </c>
-      <c r="C56" s="5">
+      <c r="C84" s="13">
         <v>6</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="D84" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E56" s="9">
-        <f>SQRT((B56-6)^2 + (C56-5)^2)</f>
+      <c r="E84" s="7">
+        <f>SQRT((B84-6)^2 + (C84-5)^2)</f>
         <v>5.0990195135927845</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="5">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" s="13">
         <v>2</v>
       </c>
-      <c r="B57" s="5">
+      <c r="B85" s="13">
         <v>2</v>
       </c>
-      <c r="C57" s="5">
+      <c r="C85" s="13">
         <v>1</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="D85" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E57" s="9">
-        <f>SQRT((B57-6)^2 + (C57-5)^2)</f>
+      <c r="E85" s="7">
+        <f>SQRT((B85-6)^2 + (C85-5)^2)</f>
         <v>5.6568542494923806</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="5">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" s="13">
         <v>19</v>
       </c>
-      <c r="B58" s="5">
+      <c r="B86" s="13">
         <v>9</v>
       </c>
-      <c r="C58" s="5">
+      <c r="C86" s="13">
         <v>10</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="D86" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E58" s="9">
-        <f>SQRT((B58-6)^2 + (C58-5)^2)</f>
+      <c r="E86" s="7">
+        <f>SQRT((B86-6)^2 + (C86-5)^2)</f>
         <v>5.8309518948453007</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="5">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" s="13">
         <v>1</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B87" s="13">
         <v>1</v>
       </c>
-      <c r="C59" s="5">
+      <c r="C87" s="13">
         <v>1</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="D87" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E59" s="9">
-        <f>SQRT((B59-6)^2 + (C59-5)^2)</f>
+      <c r="E87" s="7">
+        <f>SQRT((B87-6)^2 + (C87-5)^2)</f>
         <v>6.4031242374328485</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="5">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" s="13">
         <v>20</v>
       </c>
-      <c r="B60" s="5">
+      <c r="B88" s="13">
         <v>10</v>
       </c>
-      <c r="C60" s="5">
+      <c r="C88" s="13">
         <v>10</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D88" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E60" s="9">
-        <f>SQRT((B60-6)^2 + (C60-5)^2)</f>
+      <c r="E88" s="7">
+        <f>SQRT((B88-6)^2 + (C88-5)^2)</f>
         <v>6.4031242374328485</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A63" s="3" t="s">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B92" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B94" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B95" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C95" s="8"/>
+      <c r="D95" s="8"/>
+      <c r="E95" s="8"/>
+      <c r="F95" s="8"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B96" s="8"/>
+      <c r="C96" s="8"/>
+      <c r="D96" s="8"/>
+      <c r="E96" s="8"/>
+      <c r="F96" s="8"/>
+      <c r="G96" s="9"/>
+    </row>
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B99" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B100" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="102" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B102" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B103" s="13">
+        <v>7</v>
+      </c>
+      <c r="C103" s="13">
+        <v>7</v>
+      </c>
+      <c r="D103" s="13">
+        <v>4</v>
+      </c>
+      <c r="E103" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103" s="7">
+        <f>SQRT((C103-6)^2 + (D103-5)^2)</f>
+        <v>1.4142135623730951</v>
+      </c>
+    </row>
+    <row r="104" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B104" s="13">
+        <v>6</v>
+      </c>
+      <c r="C104" s="13">
+        <v>6</v>
+      </c>
+      <c r="D104" s="13">
+        <v>3</v>
+      </c>
+      <c r="E104" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F104" s="7">
+        <f>SQRT((C104-6)^2 + (D104-5)^2)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B105" s="13">
+        <v>5</v>
+      </c>
+      <c r="C105" s="13">
+        <v>5</v>
+      </c>
+      <c r="D105" s="13">
+        <v>3</v>
+      </c>
+      <c r="E105" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F105" s="7">
+        <f>SQRT((C105-6)^2 + (D105-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="106" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B106" s="13">
+        <v>8</v>
+      </c>
+      <c r="C106" s="13">
+        <v>8</v>
+      </c>
+      <c r="D106" s="13">
+        <v>4</v>
+      </c>
+      <c r="E106" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F106" s="7">
+        <f>SQRT((C106-6)^2 + (D106-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="107" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B107" s="13">
+        <v>9</v>
+      </c>
+      <c r="C107" s="13">
+        <v>9</v>
+      </c>
+      <c r="D107" s="13">
+        <v>5</v>
+      </c>
+      <c r="E107" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F107" s="7">
+        <f>SQRT((C107-6)^2 + (D107-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="4" t="s">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A115" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B115" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C115" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D65" s="4" t="s">
+      <c r="D115" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="5">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" s="5">
         <v>1</v>
       </c>
-      <c r="B66" s="5">
+      <c r="B116" s="5">
         <v>1</v>
-      </c>
-      <c r="C66" s="5">
-        <v>1</v>
-      </c>
-      <c r="D66" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="5">
-        <v>2</v>
-      </c>
-      <c r="B67" s="5">
-        <v>2</v>
-      </c>
-      <c r="C67" s="5">
-        <v>1</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="5">
-        <v>3</v>
-      </c>
-      <c r="B68" s="5">
-        <v>3</v>
-      </c>
-      <c r="C68" s="5">
-        <v>2</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="5">
-        <v>4</v>
-      </c>
-      <c r="B69" s="5">
-        <v>4</v>
-      </c>
-      <c r="C69" s="5">
-        <v>2</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="5">
-        <v>5</v>
-      </c>
-      <c r="B70" s="5">
-        <v>5</v>
-      </c>
-      <c r="C70" s="5">
-        <v>3</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="5">
-        <v>6</v>
-      </c>
-      <c r="B71" s="5">
-        <v>6</v>
-      </c>
-      <c r="C71" s="5">
-        <v>3</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="5">
-        <v>7</v>
-      </c>
-      <c r="B72" s="5">
-        <v>7</v>
-      </c>
-      <c r="C72" s="5">
-        <v>4</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="5">
-        <v>8</v>
-      </c>
-      <c r="B73" s="5">
-        <v>8</v>
-      </c>
-      <c r="C73" s="5">
-        <v>4</v>
-      </c>
-      <c r="D73" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="5">
-        <v>9</v>
-      </c>
-      <c r="B74" s="5">
-        <v>9</v>
-      </c>
-      <c r="C74" s="5">
-        <v>5</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="5">
-        <v>10</v>
-      </c>
-      <c r="B75" s="5">
-        <v>10</v>
-      </c>
-      <c r="C75" s="5">
-        <v>5</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="5">
-        <v>11</v>
-      </c>
-      <c r="B76" s="5">
-        <v>1</v>
-      </c>
-      <c r="C76" s="5">
-        <v>6</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="5">
-        <v>12</v>
-      </c>
-      <c r="B77" s="5">
-        <v>2</v>
-      </c>
-      <c r="C77" s="5">
-        <v>6</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="5">
-        <v>13</v>
-      </c>
-      <c r="B78" s="5">
-        <v>3</v>
-      </c>
-      <c r="C78" s="5">
-        <v>7</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="5">
-        <v>14</v>
-      </c>
-      <c r="B79" s="5">
-        <v>4</v>
-      </c>
-      <c r="C79" s="5">
-        <v>7</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="5">
-        <v>15</v>
-      </c>
-      <c r="B80" s="5">
-        <v>5</v>
-      </c>
-      <c r="C80" s="5">
-        <v>8</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="5">
-        <v>16</v>
-      </c>
-      <c r="B81" s="5">
-        <v>6</v>
-      </c>
-      <c r="C81" s="5">
-        <v>8</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="5">
-        <v>17</v>
-      </c>
-      <c r="B82" s="5">
-        <v>7</v>
-      </c>
-      <c r="C82" s="5">
-        <v>9</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="5">
-        <v>18</v>
-      </c>
-      <c r="B83" s="5">
-        <v>8</v>
-      </c>
-      <c r="C83" s="5">
-        <v>9</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="5">
-        <v>19</v>
-      </c>
-      <c r="B84" s="5">
-        <v>9</v>
-      </c>
-      <c r="C84" s="5">
-        <v>10</v>
-      </c>
-      <c r="D84" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="5">
-        <v>20</v>
-      </c>
-      <c r="B85" s="5">
-        <v>10</v>
-      </c>
-      <c r="C85" s="5">
-        <v>10</v>
-      </c>
-      <c r="D85" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A99" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E99" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" s="8">
-        <v>7</v>
-      </c>
-      <c r="B100" s="8">
-        <v>7</v>
-      </c>
-      <c r="C100" s="8">
-        <v>4</v>
-      </c>
-      <c r="D100" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E100" s="9">
-        <f>SQRT((B100-6)^2 + (C100-5)^2)</f>
-        <v>1.4142135623730951</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" s="8">
-        <v>6</v>
-      </c>
-      <c r="B101" s="8">
-        <v>6</v>
-      </c>
-      <c r="C101" s="8">
-        <v>3</v>
-      </c>
-      <c r="D101" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E101" s="9">
-        <f>SQRT((B101-6)^2 + (C101-5)^2)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="8">
-        <v>5</v>
-      </c>
-      <c r="B102" s="8">
-        <v>5</v>
-      </c>
-      <c r="C102" s="8">
-        <v>3</v>
-      </c>
-      <c r="D102" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E102" s="9">
-        <f>SQRT((B102-6)^2 + (C102-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" s="8">
-        <v>8</v>
-      </c>
-      <c r="B103" s="8">
-        <v>8</v>
-      </c>
-      <c r="C103" s="8">
-        <v>4</v>
-      </c>
-      <c r="D103" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E103" s="9">
-        <f>SQRT((B103-6)^2 + (C103-5)^2)</f>
-        <v>2.2360679774997898</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" s="5">
-        <v>14</v>
-      </c>
-      <c r="B104" s="5">
-        <v>4</v>
-      </c>
-      <c r="C104" s="5">
-        <v>7</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E104" s="9">
-        <f>SQRT((B104-6)^2 + (C104-5)^2)</f>
-        <v>2.8284271247461903</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" s="8">
-        <v>9</v>
-      </c>
-      <c r="B105" s="8">
-        <v>9</v>
-      </c>
-      <c r="C105" s="8">
-        <v>5</v>
-      </c>
-      <c r="D105" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E105" s="9">
-        <f>SQRT((B105-6)^2 + (C105-5)^2)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" s="5">
-        <v>16</v>
-      </c>
-      <c r="B106" s="5">
-        <v>6</v>
-      </c>
-      <c r="C106" s="5">
-        <v>8</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E106" s="9">
-        <f>SQRT((B106-6)^2 + (C106-5)^2)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" s="5">
-        <v>15</v>
-      </c>
-      <c r="B107" s="5">
-        <v>5</v>
-      </c>
-      <c r="C107" s="5">
-        <v>8</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E107" s="9">
-        <f>SQRT((B107-6)^2 + (C107-5)^2)</f>
-        <v>3.1622776601683795</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" s="5">
-        <v>4</v>
-      </c>
-      <c r="B108" s="5">
-        <v>4</v>
-      </c>
-      <c r="C108" s="5">
-        <v>2</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E108" s="9">
-        <f>SQRT((B108-6)^2 + (C108-5)^2)</f>
-        <v>3.6055512754639891</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" s="5">
-        <v>13</v>
-      </c>
-      <c r="B109" s="5">
-        <v>3</v>
-      </c>
-      <c r="C109" s="5">
-        <v>7</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E109" s="9">
-        <f>SQRT((B109-6)^2 + (C109-5)^2)</f>
-        <v>3.6055512754639891</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="5">
-        <v>10</v>
-      </c>
-      <c r="B110" s="5">
-        <v>10</v>
-      </c>
-      <c r="C110" s="5">
-        <v>5</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E110" s="9">
-        <f>SQRT((B110-6)^2 + (C110-5)^2)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="5">
-        <v>12</v>
-      </c>
-      <c r="B111" s="5">
-        <v>2</v>
-      </c>
-      <c r="C111" s="5">
-        <v>6</v>
-      </c>
-      <c r="D111" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E111" s="9">
-        <f>SQRT((B111-6)^2 + (C111-5)^2)</f>
-        <v>4.1231056256176606</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" s="5">
-        <v>17</v>
-      </c>
-      <c r="B112" s="5">
-        <v>7</v>
-      </c>
-      <c r="C112" s="5">
-        <v>9</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E112" s="9">
-        <f>SQRT((B112-6)^2 + (C112-5)^2)</f>
-        <v>4.1231056256176606</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="5">
-        <v>3</v>
-      </c>
-      <c r="B113" s="5">
-        <v>3</v>
-      </c>
-      <c r="C113" s="5">
-        <v>2</v>
-      </c>
-      <c r="D113" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E113" s="9">
-        <f>SQRT((B113-6)^2 + (C113-5)^2)</f>
-        <v>4.2426406871192848</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="5">
-        <v>18</v>
-      </c>
-      <c r="B114" s="5">
-        <v>8</v>
-      </c>
-      <c r="C114" s="5">
-        <v>9</v>
-      </c>
-      <c r="D114" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E114" s="9">
-        <f>SQRT((B114-6)^2 + (C114-5)^2)</f>
-        <v>4.4721359549995796</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="5">
-        <v>11</v>
-      </c>
-      <c r="B115" s="5">
-        <v>1</v>
-      </c>
-      <c r="C115" s="5">
-        <v>6</v>
-      </c>
-      <c r="D115" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E115" s="9">
-        <f>SQRT((B115-6)^2 + (C115-5)^2)</f>
-        <v>5.0990195135927845</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="5">
-        <v>2</v>
-      </c>
-      <c r="B116" s="5">
-        <v>2</v>
       </c>
       <c r="C116" s="5">
         <v>1</v>
@@ -6009,71 +5484,661 @@
       <c r="D116" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E116" s="9">
-        <f>SQRT((B116-6)^2 + (C116-5)^2)</f>
-        <v>5.6568542494923806</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="5">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B117" s="5">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C117" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E117" s="9">
-        <f>SQRT((B117-6)^2 + (C117-5)^2)</f>
-        <v>5.8309518948453007</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B118" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C118" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E118" s="9">
-        <f>SQRT((B118-6)^2 + (C118-5)^2)</f>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A119" s="5">
+        <v>4</v>
+      </c>
+      <c r="B119" s="5">
+        <v>4</v>
+      </c>
+      <c r="C119" s="5">
+        <v>2</v>
+      </c>
+      <c r="D119" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A120" s="5">
+        <v>5</v>
+      </c>
+      <c r="B120" s="5">
+        <v>5</v>
+      </c>
+      <c r="C120" s="5">
+        <v>3</v>
+      </c>
+      <c r="D120" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A121" s="5">
+        <v>6</v>
+      </c>
+      <c r="B121" s="5">
+        <v>6</v>
+      </c>
+      <c r="C121" s="5">
+        <v>3</v>
+      </c>
+      <c r="D121" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A122" s="5">
+        <v>7</v>
+      </c>
+      <c r="B122" s="5">
+        <v>7</v>
+      </c>
+      <c r="C122" s="5">
+        <v>4</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A123" s="5">
+        <v>8</v>
+      </c>
+      <c r="B123" s="5">
+        <v>8</v>
+      </c>
+      <c r="C123" s="5">
+        <v>4</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A124" s="5">
+        <v>9</v>
+      </c>
+      <c r="B124" s="5">
+        <v>9</v>
+      </c>
+      <c r="C124" s="5">
+        <v>5</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A125" s="5">
+        <v>10</v>
+      </c>
+      <c r="B125" s="5">
+        <v>10</v>
+      </c>
+      <c r="C125" s="5">
+        <v>5</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A126" s="5">
+        <v>11</v>
+      </c>
+      <c r="B126" s="5">
+        <v>1</v>
+      </c>
+      <c r="C126" s="5">
+        <v>6</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A127" s="5">
+        <v>12</v>
+      </c>
+      <c r="B127" s="5">
+        <v>2</v>
+      </c>
+      <c r="C127" s="5">
+        <v>6</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A128" s="5">
+        <v>13</v>
+      </c>
+      <c r="B128" s="5">
+        <v>3</v>
+      </c>
+      <c r="C128" s="5">
+        <v>7</v>
+      </c>
+      <c r="D128" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A129" s="5">
+        <v>14</v>
+      </c>
+      <c r="B129" s="5">
+        <v>4</v>
+      </c>
+      <c r="C129" s="5">
+        <v>7</v>
+      </c>
+      <c r="D129" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A130" s="5">
+        <v>15</v>
+      </c>
+      <c r="B130" s="5">
+        <v>5</v>
+      </c>
+      <c r="C130" s="5">
+        <v>8</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A131" s="5">
+        <v>16</v>
+      </c>
+      <c r="B131" s="5">
+        <v>6</v>
+      </c>
+      <c r="C131" s="5">
+        <v>8</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A132" s="5">
+        <v>17</v>
+      </c>
+      <c r="B132" s="5">
+        <v>7</v>
+      </c>
+      <c r="C132" s="5">
+        <v>9</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A133" s="5">
+        <v>18</v>
+      </c>
+      <c r="B133" s="5">
+        <v>8</v>
+      </c>
+      <c r="C133" s="5">
+        <v>9</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A134" s="5">
+        <v>19</v>
+      </c>
+      <c r="B134" s="5">
+        <v>9</v>
+      </c>
+      <c r="C134" s="5">
+        <v>10</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A135" s="5">
+        <v>20</v>
+      </c>
+      <c r="B135" s="5">
+        <v>10</v>
+      </c>
+      <c r="C135" s="5">
+        <v>10</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="149" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B149" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="151" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B151" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D151" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="152" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B152" s="13">
+        <v>7</v>
+      </c>
+      <c r="C152" s="13">
+        <v>7</v>
+      </c>
+      <c r="D152" s="13">
+        <v>4</v>
+      </c>
+      <c r="E152" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F152" s="7">
+        <f>SQRT((C152-6)^2 + (D152-5)^2)</f>
+        <v>1.4142135623730951</v>
+      </c>
+    </row>
+    <row r="153" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B153" s="13">
+        <v>6</v>
+      </c>
+      <c r="C153" s="13">
+        <v>6</v>
+      </c>
+      <c r="D153" s="13">
+        <v>3</v>
+      </c>
+      <c r="E153" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F153" s="7">
+        <f>SQRT((C153-6)^2 + (D153-5)^2)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="154" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B154" s="13">
+        <v>5</v>
+      </c>
+      <c r="C154" s="13">
+        <v>5</v>
+      </c>
+      <c r="D154" s="13">
+        <v>3</v>
+      </c>
+      <c r="E154" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F154" s="7">
+        <f>SQRT((C154-6)^2 + (D154-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="155" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B155" s="13">
+        <v>8</v>
+      </c>
+      <c r="C155" s="13">
+        <v>8</v>
+      </c>
+      <c r="D155" s="13">
+        <v>4</v>
+      </c>
+      <c r="E155" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F155" s="7">
+        <f>SQRT((C155-6)^2 + (D155-5)^2)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="156" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B156" s="13">
+        <v>14</v>
+      </c>
+      <c r="C156" s="13">
+        <v>4</v>
+      </c>
+      <c r="D156" s="13">
+        <v>7</v>
+      </c>
+      <c r="E156" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F156" s="7">
+        <f>SQRT((C156-6)^2 + (D156-5)^2)</f>
+        <v>2.8284271247461903</v>
+      </c>
+    </row>
+    <row r="157" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B157" s="13">
+        <v>9</v>
+      </c>
+      <c r="C157" s="13">
+        <v>9</v>
+      </c>
+      <c r="D157" s="13">
+        <v>5</v>
+      </c>
+      <c r="E157" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F157" s="7">
+        <f>SQRT((C157-6)^2 + (D157-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="158" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B158" s="13">
+        <v>16</v>
+      </c>
+      <c r="C158" s="13">
+        <v>6</v>
+      </c>
+      <c r="D158" s="13">
+        <v>8</v>
+      </c>
+      <c r="E158" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F158" s="7">
+        <f>SQRT((C158-6)^2 + (D158-5)^2)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="159" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B159" s="13">
+        <v>15</v>
+      </c>
+      <c r="C159" s="13">
+        <v>5</v>
+      </c>
+      <c r="D159" s="13">
+        <v>8</v>
+      </c>
+      <c r="E159" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F159" s="7">
+        <f>SQRT((C159-6)^2 + (D159-5)^2)</f>
+        <v>3.1622776601683795</v>
+      </c>
+    </row>
+    <row r="160" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B160" s="13">
+        <v>4</v>
+      </c>
+      <c r="C160" s="13">
+        <v>4</v>
+      </c>
+      <c r="D160" s="13">
+        <v>2</v>
+      </c>
+      <c r="E160" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F160" s="7">
+        <f>SQRT((C160-6)^2 + (D160-5)^2)</f>
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="161" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B161" s="13">
+        <v>13</v>
+      </c>
+      <c r="C161" s="13">
+        <v>3</v>
+      </c>
+      <c r="D161" s="13">
+        <v>7</v>
+      </c>
+      <c r="E161" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F161" s="7">
+        <f>SQRT((C161-6)^2 + (D161-5)^2)</f>
+        <v>3.6055512754639891</v>
+      </c>
+    </row>
+    <row r="162" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B162" s="13">
+        <v>10</v>
+      </c>
+      <c r="C162" s="13">
+        <v>10</v>
+      </c>
+      <c r="D162" s="13">
+        <v>5</v>
+      </c>
+      <c r="E162" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F162" s="7">
+        <f>SQRT((C162-6)^2 + (D162-5)^2)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="163" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B163" s="13">
+        <v>12</v>
+      </c>
+      <c r="C163" s="13">
+        <v>2</v>
+      </c>
+      <c r="D163" s="13">
+        <v>6</v>
+      </c>
+      <c r="E163" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F163" s="7">
+        <f>SQRT((C163-6)^2 + (D163-5)^2)</f>
+        <v>4.1231056256176606</v>
+      </c>
+    </row>
+    <row r="164" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B164" s="13">
+        <v>17</v>
+      </c>
+      <c r="C164" s="13">
+        <v>7</v>
+      </c>
+      <c r="D164" s="13">
+        <v>9</v>
+      </c>
+      <c r="E164" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F164" s="7">
+        <f>SQRT((C164-6)^2 + (D164-5)^2)</f>
+        <v>4.1231056256176606</v>
+      </c>
+    </row>
+    <row r="165" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B165" s="13">
+        <v>3</v>
+      </c>
+      <c r="C165" s="13">
+        <v>3</v>
+      </c>
+      <c r="D165" s="13">
+        <v>2</v>
+      </c>
+      <c r="E165" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F165" s="7">
+        <f>SQRT((C165-6)^2 + (D165-5)^2)</f>
+        <v>4.2426406871192848</v>
+      </c>
+    </row>
+    <row r="166" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B166" s="13">
+        <v>18</v>
+      </c>
+      <c r="C166" s="13">
+        <v>8</v>
+      </c>
+      <c r="D166" s="13">
+        <v>9</v>
+      </c>
+      <c r="E166" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F166" s="7">
+        <f>SQRT((C166-6)^2 + (D166-5)^2)</f>
+        <v>4.4721359549995796</v>
+      </c>
+    </row>
+    <row r="167" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B167" s="13">
+        <v>11</v>
+      </c>
+      <c r="C167" s="13">
+        <v>1</v>
+      </c>
+      <c r="D167" s="13">
+        <v>6</v>
+      </c>
+      <c r="E167" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F167" s="7">
+        <f>SQRT((C167-6)^2 + (D167-5)^2)</f>
+        <v>5.0990195135927845</v>
+      </c>
+    </row>
+    <row r="168" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B168" s="13">
+        <v>2</v>
+      </c>
+      <c r="C168" s="13">
+        <v>2</v>
+      </c>
+      <c r="D168" s="13">
+        <v>1</v>
+      </c>
+      <c r="E168" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F168" s="7">
+        <f>SQRT((C168-6)^2 + (D168-5)^2)</f>
+        <v>5.6568542494923806</v>
+      </c>
+    </row>
+    <row r="169" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B169" s="13">
+        <v>19</v>
+      </c>
+      <c r="C169" s="13">
+        <v>9</v>
+      </c>
+      <c r="D169" s="13">
+        <v>10</v>
+      </c>
+      <c r="E169" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F169" s="7">
+        <f>SQRT((C169-6)^2 + (D169-5)^2)</f>
+        <v>5.8309518948453007</v>
+      </c>
+    </row>
+    <row r="170" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B170" s="13">
+        <v>1</v>
+      </c>
+      <c r="C170" s="13">
+        <v>1</v>
+      </c>
+      <c r="D170" s="13">
+        <v>1</v>
+      </c>
+      <c r="E170" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F170" s="7">
+        <f>SQRT((C170-6)^2 + (D170-5)^2)</f>
         <v>6.4031242374328485</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="5">
+    <row r="171" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B171" s="13">
         <v>20</v>
       </c>
-      <c r="B119" s="5">
+      <c r="C171" s="13">
         <v>10</v>
       </c>
-      <c r="C119" s="5">
+      <c r="D171" s="13">
         <v>10</v>
       </c>
-      <c r="D119" s="5" t="s">
+      <c r="E171" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E119" s="9">
-        <f>SQRT((B119-6)^2 + (C119-5)^2)</f>
+      <c r="F171" s="7">
+        <f>SQRT((C171-6)^2 + (D171-5)^2)</f>
         <v>6.4031242374328485</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="H9:L28">
-    <sortCondition ref="L28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A36:E55">
+    <sortCondition ref="E55"/>
   </sortState>
   <mergeCells count="1">
-    <mergeCell ref="I33:N34"/>
+    <mergeCell ref="B95:G96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>